<commit_message>
updated logfile upto october 15
</commit_message>
<xml_diff>
--- a/logfile.xlsx
+++ b/logfile.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/109592e82ad92d31/Desktop/SwastyaAI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="140" documentId="8_{E83579EE-C5B4-4637-9CC9-5AB53764051F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A8546A8-EC50-4BC3-9831-797FF4E7EFAD}"/>
+  <xr:revisionPtr revIDLastSave="186" documentId="8_{E83579EE-C5B4-4637-9CC9-5AB53764051F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{54E35EA1-E906-4CD1-874F-17C1AA7A37AE}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{A1A36BEB-C7EC-4B99-9D9A-72C12A907096}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="21">
   <si>
     <t>Log File of SwasthyaAI Research</t>
   </si>
@@ -80,10 +80,28 @@
     <t xml:space="preserve">discuss about topic </t>
   </si>
   <si>
-    <t>Training ,guide to Binod and Deepa</t>
-  </si>
-  <si>
     <t>run dr.html,show DR prediction result</t>
+  </si>
+  <si>
+    <t>Oct 9-15</t>
+  </si>
+  <si>
+    <t>Training ,guide to Binod and Deepa,add effiocientnetB0 for seed 42,123 and 2024</t>
+  </si>
+  <si>
+    <t>add quantitative button perfomance of dr and close its issue</t>
+  </si>
+  <si>
+    <t>created 6 issues of dr,dr qualitative grid image</t>
+  </si>
+  <si>
+    <t>center  sepeartion of dr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">push ppt of dr details </t>
+  </si>
+  <si>
+    <t>create new branch named binod and add eye labeler app(right/left) and assests</t>
   </si>
 </sst>
 </file>
@@ -202,7 +220,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
@@ -210,11 +228,41 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -223,22 +271,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" indent="2"/>
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -255,6 +288,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -575,140 +612,151 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6983F01E-A41D-440F-A806-34677778C9B3}">
   <dimension ref="A2:I28"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.7109375" style="10" customWidth="1"/>
-    <col min="2" max="2" width="25.85546875" style="10" customWidth="1"/>
-    <col min="3" max="3" width="34.28515625" style="10" customWidth="1"/>
-    <col min="4" max="4" width="20.42578125" style="10" customWidth="1"/>
-    <col min="5" max="6" width="9.140625" style="10" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="10"/>
+    <col min="1" max="1" width="22.7109375" style="4" customWidth="1"/>
+    <col min="2" max="2" width="25.85546875" style="4" customWidth="1"/>
+    <col min="3" max="3" width="75.5703125" style="4" customWidth="1"/>
+    <col min="4" max="4" width="20.42578125" style="4" customWidth="1"/>
+    <col min="5" max="6" width="9.140625" style="4" customWidth="1"/>
+    <col min="7" max="16384" width="10.7109375" style="4"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:9" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
     </row>
     <row r="4" spans="1:9" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="7" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="8"/>
-      <c r="B6" s="2" t="s">
+      <c r="A6" s="11"/>
+      <c r="B6" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="6"/>
+      <c r="F6" s="5"/>
+      <c r="I6" s="2"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="11"/>
+      <c r="B7" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="6"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="11"/>
+      <c r="B8" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="2"/>
-      <c r="F6" s="12"/>
-      <c r="I6" s="2"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="8"/>
-      <c r="B7" s="2" t="s">
+      <c r="D8" s="6"/>
+    </row>
+    <row r="9" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="12"/>
+      <c r="B9" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="6"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="6"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="15"/>
+      <c r="B11" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11" s="6"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="15"/>
+      <c r="B12" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" s="2"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="8"/>
-      <c r="B8" s="2" t="s">
+      <c r="C12" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="17"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="15"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="16"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="15"/>
+      <c r="B14" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D8" s="2"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="9"/>
-      <c r="B9" s="2" t="s">
+      <c r="C14" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D14" s="6"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="16"/>
+      <c r="B15" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D9" s="2"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="4"/>
-      <c r="B10" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="5"/>
-      <c r="B11" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="5"/>
-      <c r="B12" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="5"/>
-      <c r="B13" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="6"/>
-      <c r="B14" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
+      <c r="C15" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D15" s="6"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
     </row>
@@ -785,10 +833,13 @@
       <c r="D28" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="6">
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="A5:A9"/>
-    <mergeCell ref="A10:A14"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="A11:A15"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="D12:D13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
logfile upto october 22
</commit_message>
<xml_diff>
--- a/logfile.xlsx
+++ b/logfile.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/109592e82ad92d31/Desktop/SwastyaAI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="186" documentId="8_{E83579EE-C5B4-4637-9CC9-5AB53764051F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{54E35EA1-E906-4CD1-874F-17C1AA7A37AE}"/>
+  <xr:revisionPtr revIDLastSave="265" documentId="8_{E83579EE-C5B4-4637-9CC9-5AB53764051F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F3186203-4AFE-41BE-9170-7A52400FCA6B}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{A1A36BEB-C7EC-4B99-9D9A-72C12A907096}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="27">
   <si>
     <t>Log File of SwasthyaAI Research</t>
   </si>
@@ -95,13 +95,31 @@
     <t>created 6 issues of dr,dr qualitative grid image</t>
   </si>
   <si>
+    <t xml:space="preserve">push ppt of dr details </t>
+  </si>
+  <si>
+    <t>create new branch named binod and add eye labeler app(right/left) and assests</t>
+  </si>
+  <si>
+    <t>solve vercel issue</t>
+  </si>
+  <si>
+    <t>added grade library ,gradewise details of DR,Dropdown edited of Select Model</t>
+  </si>
+  <si>
     <t>center  sepeartion of dr</t>
   </si>
   <si>
-    <t xml:space="preserve">push ppt of dr details </t>
-  </si>
-  <si>
-    <t>create new branch named binod and add eye labeler app(right/left) and assests</t>
+    <t>Oct16-22</t>
+  </si>
+  <si>
+    <t>upload combined csv of dr patient id,left/right+center by Anisha,Bikram and Binod,pyproject.toml added</t>
+  </si>
+  <si>
+    <t>efficinent net b3 training  for aptos and multimodal dataset  csv given by Bikram</t>
+  </si>
+  <si>
+    <t>laptop problem</t>
   </si>
 </sst>
 </file>
@@ -220,7 +238,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
@@ -228,49 +246,43 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -614,174 +626,197 @@
   <dimension ref="A2:I28"/>
   <sheetFormatPr defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.7109375" style="4" customWidth="1"/>
-    <col min="2" max="2" width="25.85546875" style="4" customWidth="1"/>
-    <col min="3" max="3" width="75.5703125" style="4" customWidth="1"/>
-    <col min="4" max="4" width="20.42578125" style="4" customWidth="1"/>
-    <col min="5" max="6" width="9.140625" style="4" customWidth="1"/>
-    <col min="7" max="16384" width="10.7109375" style="4"/>
+    <col min="1" max="1" width="22.7109375" style="3" customWidth="1"/>
+    <col min="2" max="2" width="25.85546875" style="3" customWidth="1"/>
+    <col min="3" max="3" width="89.140625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="20.42578125" style="3" customWidth="1"/>
+    <col min="5" max="6" width="9.140625" style="3" customWidth="1"/>
+    <col min="7" max="16384" width="10.7109375" style="3"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:9" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
     </row>
     <row r="4" spans="1:9" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="6" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="11"/>
-      <c r="B6" s="8" t="s">
+      <c r="A6" s="9"/>
+      <c r="B6" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="6"/>
-      <c r="F6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="F6" s="4"/>
       <c r="I6" s="2"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="11"/>
-      <c r="B7" s="8" t="s">
+      <c r="A7" s="9"/>
+      <c r="B7" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="6"/>
+      <c r="D7" s="5"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="11"/>
-      <c r="B8" s="8" t="s">
+      <c r="A8" s="9"/>
+      <c r="B8" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="6"/>
+      <c r="D8" s="5"/>
     </row>
     <row r="9" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="12"/>
-      <c r="B9" s="8" t="s">
+      <c r="A9" s="10"/>
+      <c r="B9" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="6"/>
+      <c r="D9" s="5"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="5"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="9"/>
+      <c r="B11" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11" s="5"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="9"/>
+      <c r="B12" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" s="14"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="9"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="15"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="9"/>
+      <c r="B14" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D14" s="5"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="10"/>
+      <c r="B15" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="6"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="15"/>
-      <c r="B11" s="8" t="s">
+      <c r="D15" s="5"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" s="2"/>
+    </row>
+    <row r="17" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="9"/>
+      <c r="B17" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="D11" s="6"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="15"/>
-      <c r="B12" s="13" t="s">
+      <c r="C17" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D17" s="2"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="9"/>
+      <c r="B18" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="D12" s="17"/>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="15"/>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="16"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="15"/>
-      <c r="B14" s="8" t="s">
+      <c r="C18" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D18" s="2"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="9"/>
+      <c r="B19" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C14" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="D14" s="6"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="16"/>
-      <c r="B15" s="8" t="s">
+      <c r="C19" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D19" s="2"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="10"/>
+      <c r="B20" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D15" s="6"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
+      <c r="C20" s="2" t="s">
+        <v>26</v>
+      </c>
       <c r="D20" s="2"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -833,11 +868,12 @@
       <c r="D28" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
+    <mergeCell ref="A16:A20"/>
+    <mergeCell ref="A10:A15"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="A5:A9"/>
     <mergeCell ref="C12:C13"/>
-    <mergeCell ref="A11:A15"/>
     <mergeCell ref="B12:B13"/>
     <mergeCell ref="D12:D13"/>
   </mergeCells>

</xml_diff>

<commit_message>
logfile of this week
</commit_message>
<xml_diff>
--- a/logfile.xlsx
+++ b/logfile.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/109592e82ad92d31/Desktop/SwastyaAI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="265" documentId="8_{E83579EE-C5B4-4637-9CC9-5AB53764051F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F3186203-4AFE-41BE-9170-7A52400FCA6B}"/>
+  <xr:revisionPtr revIDLastSave="271" documentId="8_{E83579EE-C5B4-4637-9CC9-5AB53764051F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{71635161-AE71-4B47-84D2-EFC820E9B266}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{A1A36BEB-C7EC-4B99-9D9A-72C12A907096}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="29">
   <si>
     <t>Log File of SwasthyaAI Research</t>
   </si>
@@ -119,7 +119,13 @@
     <t>efficinent net b3 training  for aptos and multimodal dataset  csv given by Bikram</t>
   </si>
   <si>
-    <t>laptop problem</t>
+    <t>computer problem</t>
+  </si>
+  <si>
+    <t>Oct 23-29</t>
+  </si>
+  <si>
+    <t>language translation work</t>
   </si>
 </sst>
 </file>
@@ -820,9 +826,15 @@
       <c r="D20" s="2"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
+      <c r="A21" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>28</v>
+      </c>
       <c r="D21" s="2"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>